<commit_message>
EPBDS-7164 Show transposed Run, keyed Data and referencing Test tables in Example 4
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/1-Data-Model/DataTables.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/1-Data-Model/DataTables.xlsx
@@ -1549,9 +1549,9 @@
     <mergeCell ref="B21:I21"/>
     <mergeCell ref="B48:C48"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B4:I4"/>
     <mergeCell ref="B32:G32"/>
     <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B4:I4"/>
     <mergeCell ref="B37:I37"/>
     <mergeCell ref="B13:F13"/>
   </mergeCells>
@@ -1566,7 +1566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I65"/>
+  <dimension ref="B2:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -2255,17 +2255,200 @@
         </is>
       </c>
     </row>
+    <row r="67" ht="16.5" customHeight="1">
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>A transposed data table keeps both keys: "_PK_" in the first row and "&gt;table" in the column next to the field names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Data Employee managers</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="n"/>
+      <c r="D69" s="9" t="n"/>
+      <c r="E69" s="9" t="n"/>
+      <c r="F69" s="7" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>_PK_</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="n"/>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="n"/>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>Eve</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>Finn</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>store</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>&gt;stores</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Store</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="n"/>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Method String ManagerCity(Integer index)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>return managers[index].store.city;</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Test ManagerCity ManagerCityTest</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="n"/>
+    </row>
+    <row r="79">
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Index</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>Denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="16">
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B21:I21"/>
     <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B21:I21"/>
-    <mergeCell ref="B44:C44"/>
     <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B69:F69"/>
     <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B78:C78"/>
     <mergeCell ref="B38:I38"/>
     <mergeCell ref="B51:I51"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B67:I67"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B62:G62"/>
     <mergeCell ref="B53:C53"/>

</xml_diff>